<commit_message>
feat: implement job automation core, project configuration, and document generation pipeline
</commit_message>
<xml_diff>
--- a/output/Job_Matching_Updated.xlsx
+++ b/output/Job_Matching_Updated.xlsx
@@ -668,20 +668,20 @@
         </is>
       </c>
       <c r="W2">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\BMW_Group_Intern_Quantum_Computing_Applications_wmx.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\BMW_Group_Intern_Quantum_Computing_Applications_wmx.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X2">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\BMW_Group_Intern_Quantum_Computing_Applications_wmx.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\BMW_Group_Intern_Quantum_Computing_Applications_wmx.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y2">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\BMW_Group_Intern_Quantum_Computing_Applications_wmx_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\BMW_Group_Intern_Quantum_Computing_Applications_wmx_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:28.852009</t>
+          <t>2026-06-28T09:17:35.121832</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>mpi, openmp, fortran</t>
+          <t>fortran</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -763,11 +763,11 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Overall match: 86%; Education: 80%, Skills: 100%, Programming: 73%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, openmp, fortran</t>
+          <t>Overall match: 89%; Education: 80%, Skills: 100%, Programming: 73%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: fortran</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -781,20 +781,20 @@
         </is>
       </c>
       <c r="W3">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Karlsruher_Institut_für_Technologie_KIT_Helmholtz__Research_Software_Engineer_fmd_HPC_RSE.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Karlsruher_Institut_für_Technologie_KIT_Helmholtz__Research_Software_Engineer_fmd_HPC_RSE.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X3">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Karlsruher_Institut_für_Technologie_KIT_Helmholtz__Research_Software_Engineer_fmd_HPC_RSE.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Karlsruher_Institut_für_Technologie_KIT_Helmholtz__Research_Software_Engineer_fmd_HPC_RSE.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y3">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Karlsruher_Institut_für_Technologie_KIT_Helmholtz__Research_Software_Engineer_fmd_HPC_RSE_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Karlsruher_Institut_für_Technologie_KIT_Helmholtz__Research_Software_Engineer_fmd_HPC_RSE_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:29.070486</t>
+          <t>2026-06-28T09:17:34.993934</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>mpi, openmp, fortran</t>
+          <t>fortran</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -876,11 +876,11 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Overall match: 86%; Education: 80%, Skills: 100%, Programming: 73%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, openmp, fortran</t>
+          <t>Overall match: 89%; Education: 80%, Skills: 100%, Programming: 73%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: fortran</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -894,20 +894,20 @@
         </is>
       </c>
       <c r="W4">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Forschungszentrum_Jülich_JSC_Research_Software_Engineer.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Forschungszentrum_Jülich_JSC_Research_Software_Engineer.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X4">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Forschungszentrum_Jülich_JSC_Research_Software_Engineer.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Forschungszentrum_Jülich_JSC_Research_Software_Engineer.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y4">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Forschungszentrum_Jülich_JSC_Research_Software_Engineer_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Forschungszentrum_Jülich_JSC_Research_Software_Engineer_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:28.816015</t>
+          <t>2026-06-28T09:17:35.088359</t>
         </is>
       </c>
     </row>
@@ -963,11 +963,7 @@
           <t>HPC, AI, Python, Scientific Computing, Optimization Methods, System Design, Training interest</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>cuda</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>Research Position (TV-L 13)</t>
@@ -989,11 +985,11 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Overall match: 85%; Education: 70%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: cuda</t>
+          <t>Overall match: 88%; Education: 70%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1007,20 +1003,20 @@
         </is>
       </c>
       <c r="W5">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\University_of_Stuttgart_HLRS_SFB_1313_Research_Scientist_with_focus_on_HPC_AI_and_traini.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\University_of_Stuttgart_HLRS_SFB_1313_Research_Scientist_with_focus_on_HPC_AI_and_traini.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X5">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\University_of_Stuttgart_HLRS_SFB_1313_Research_Scientist_with_focus_on_HPC_AI_and_traini.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\University_of_Stuttgart_HLRS_SFB_1313_Research_Scientist_with_focus_on_HPC_AI_and_traini.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y5">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\University_of_Stuttgart_HLRS_SFB_1313_Research_Scientist_with_focus_on_HPC_AI_and_traini_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\University_of_Stuttgart_HLRS_SFB_1313_Research_Scientist_with_focus_on_HPC_AI_and_traini_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:28.701206</t>
+          <t>2026-06-28T09:17:35.045322</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1074,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>mpi, openmp, cuda, fortran</t>
+          <t>fortran</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1102,11 +1098,11 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Overall match: 77%; Education: 50%, Skills: 100%, Programming: 73%; Research: 80%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, openmp, cuda, fortran</t>
+          <t>Overall match: 80%; Education: 50%, Skills: 100%, Programming: 73%; Research: 100%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: fortran</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1120,20 +1116,20 @@
         </is>
       </c>
       <c r="W6">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\German_Climate_Computing_Center_DKRZ_Research_Software_Engineer_Coupled_Climate_Models_.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\German_Climate_Computing_Center_DKRZ_Research_Software_Engineer_Coupled_Climate_Models_.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X6">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\German_Climate_Computing_Center_DKRZ_Research_Software_Engineer_Coupled_Climate_Models_.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\German_Climate_Computing_Center_DKRZ_Research_Software_Engineer_Coupled_Climate_Models_.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y6">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\German_Climate_Computing_Center_DKRZ_Research_Software_Engineer_Coupled_Climate_Models__CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\German_Climate_Computing_Center_DKRZ_Research_Software_Engineer_Coupled_Climate_Models__CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:33.375791</t>
+          <t>2026-06-28T09:17:39.263757</t>
         </is>
       </c>
     </row>
@@ -1189,11 +1185,7 @@
           <t>HPC, Python, Linux, Git, Workflow concepts, Scientific Computing</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>docker</t>
-        </is>
-      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>Research Engineer</t>
@@ -1215,11 +1207,11 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
-        <v>76.5</v>
+        <v>80.5</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Overall match: 76%; Education: 40%, Skills: 90%, Programming: 100%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: docker</t>
+          <t>Overall match: 80%; Education: 40%, Skills: 100%, Programming: 100%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1233,20 +1225,20 @@
         </is>
       </c>
       <c r="W7">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Barcelona_Supercomputing_Center_BSC_CNS_HPC_Workflows_Engineer_RE1_RE2.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Barcelona_Supercomputing_Center_BSC_CNS_HPC_Workflows_Engineer_RE1_RE2.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X7">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Barcelona_Supercomputing_Center_BSC_CNS_HPC_Workflows_Engineer_RE1_RE2.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Barcelona_Supercomputing_Center_BSC_CNS_HPC_Workflows_Engineer_RE1_RE2.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y7">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Barcelona_Supercomputing_Center_BSC_CNS_HPC_Workflows_Engineer_RE1_RE2_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Barcelona_Supercomputing_Center_BSC_CNS_HPC_Workflows_Engineer_RE1_RE2_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:33.394654</t>
+          <t>2026-06-28T09:17:39.212209</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1572,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>slurm, lustre</t>
+          <t>lustre</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1608,7 +1600,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Overall match: 82%; Education: 50%, Skills: 100%, Programming: 100%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background; Missing: slurm, lustre</t>
+          <t>Overall match: 82%; Education: 50%, Skills: 100%, Programming: 100%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background; Missing: lustre</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1622,20 +1614,20 @@
         </is>
       </c>
       <c r="W11">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Zuse_Institute_Berlin_ZIB_System_Administrator_HPC_wmd.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Zuse_Institute_Berlin_ZIB_System_Administrator_HPC_wmd.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X11">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Zuse_Institute_Berlin_ZIB_System_Administrator_HPC_wmd.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Zuse_Institute_Berlin_ZIB_System_Administrator_HPC_wmd.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y11">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Zuse_Institute_Berlin_ZIB_System_Administrator_HPC_wmd_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Zuse_Institute_Berlin_ZIB_System_Administrator_HPC_wmd_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:33.418461</t>
+          <t>2026-06-28T09:17:39.301010</t>
         </is>
       </c>
     </row>
@@ -1691,11 +1683,7 @@
           <t>HPC, Deep Learning, Python, C++, GPU concepts, Performance Optimization</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>mpi, cuda</t>
-        </is>
-      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -1717,11 +1705,11 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Overall match: 79%; Education: 40%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, cuda</t>
+          <t>Overall match: 82%; Education: 40%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1735,20 +1723,20 @@
         </is>
       </c>
       <c r="W12">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\NVIDIA_Senior_Software_Architect_Deep_Learning_and_HPC_Co.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\NVIDIA_Senior_Software_Architect_Deep_Learning_and_HPC_Co.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X12">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\NVIDIA_Senior_Software_Architect_Deep_Learning_and_HPC_Co.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\NVIDIA_Senior_Software_Architect_Deep_Learning_and_HPC_Co.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y12">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\NVIDIA_Senior_Software_Architect_Deep_Learning_and_HPC_Co_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\NVIDIA_Senior_Software_Architect_Deep_Learning_and_HPC_Co_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:33.474394</t>
+          <t>2026-06-28T09:17:39.381387</t>
         </is>
       </c>
     </row>
@@ -1804,11 +1792,7 @@
           <t>HPC, GPU, Python, C/C++, Scientific Computing, Parallel Computing, Research, Optimization</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>cuda</t>
-        </is>
-      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>PhD (3 years, 75% TVöD E13)</t>
@@ -1830,11 +1814,11 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Overall match: 88%; Education: 70%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: cuda</t>
+          <t>Overall match: 91%; Education: 70%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1848,20 +1832,20 @@
         </is>
       </c>
       <c r="W13">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_PhD_Student_fmd_for_HPCGPU_Computing.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_PhD_Student_fmd_for_HPCGPU_Computing.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X13">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_PhD_Student_fmd_for_HPCGPU_Computing.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_PhD_Student_fmd_for_HPCGPU_Computing.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y13">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_PhD_Student_fmd_for_HPCGPU_Computing_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_PhD_Student_fmd_for_HPCGPU_Computing_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:37.511395</t>
+          <t>2026-06-28T09:17:43.382323</t>
         </is>
       </c>
     </row>
@@ -1917,11 +1901,7 @@
           <t>HPC, GPU, Python, C/C++, Scientific Computing, Research, Publications</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>mpi, openmp, cuda</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>Postdoc</t>
@@ -1943,11 +1923,11 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Overall match: 82%; Education: 40%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background; Missing: mpi, openmp, cuda</t>
+          <t>Overall match: 85%; Education: 40%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1961,20 +1941,20 @@
         </is>
       </c>
       <c r="W14">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_Postdoc_fmd_for_HPCGPU_Computing.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_Postdoc_fmd_for_HPCGPU_Computing.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X14">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_Postdoc_fmd_for_HPCGPU_Computing.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_Postdoc_fmd_for_HPCGPU_Computing.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y14">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_Postdoc_fmd_for_HPCGPU_Computing_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Helmholtz_Zentrum_Dresden_Rossendorf_HZDR_CASUS_Postdoc_fmd_for_HPCGPU_Computing_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:37.534068</t>
+          <t>2026-06-28T09:17:43.405985</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2012,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>kubernetes, docker</t>
+          <t>kubernetes</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2056,11 +2036,11 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
-        <v>75.5</v>
+        <v>79.5</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Overall match: 76%; Education: 50%, Skills: 90%, Programming: 100%; Research: 70%, Experience: 40%; Strengths: Python programming, HPC background; Missing: kubernetes, docker</t>
+          <t>Overall match: 80%; Education: 50%, Skills: 100%, Programming: 100%; Research: 70%, Experience: 40%; Strengths: Python programming, HPC background; Missing: kubernetes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2074,20 +2054,20 @@
         </is>
       </c>
       <c r="W15">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Mistral_AI_Systems_Engineer_HPC.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Mistral_AI_Systems_Engineer_HPC.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X15">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Mistral_AI_Systems_Engineer_HPC.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Mistral_AI_Systems_Engineer_HPC.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y15">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Mistral_AI_Systems_Engineer_HPC_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Mistral_AI_Systems_Engineer_HPC_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:37.725618</t>
+          <t>2026-06-28T09:17:43.624486</t>
         </is>
       </c>
     </row>
@@ -2143,11 +2123,7 @@
           <t>HPC, System Software, Linux, Python, C, Research interest</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>mpi, openmp</t>
-        </is>
-      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>Research</t>
@@ -2169,11 +2145,11 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Overall match: 81%; Education: 70%, Skills: 100%, Programming: 73%; Research: 80%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, openmp</t>
+          <t>Overall match: 84%; Education: 70%, Skills: 100%, Programming: 73%; Research: 100%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2187,20 +2163,20 @@
         </is>
       </c>
       <c r="W16">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Technische_Universität_Dresden_Research_Associate_HPC_System_Software_Engineer_mf.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Technische_Universität_Dresden_Research_Associate_HPC_System_Software_Engineer_mf.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X16">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Technische_Universität_Dresden_Research_Associate_HPC_System_Software_Engineer_mf.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Technische_Universität_Dresden_Research_Associate_HPC_System_Software_Engineer_mf.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y16">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Technische_Universität_Dresden_Research_Associate_HPC_System_Software_Engineer_mf_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Technische_Universität_Dresden_Research_Associate_HPC_System_Software_Engineer_mf_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:37.656148</t>
+          <t>2026-06-28T09:17:43.692743</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2234,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>mpi, fortran</t>
+          <t>fortran</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2286,7 +2262,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Overall match: 78%; Education: 50%, Skills: 100%, Programming: 73%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, fortran</t>
+          <t>Overall match: 78%; Education: 50%, Skills: 100%, Programming: 73%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: fortran</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2300,20 +2276,20 @@
         </is>
       </c>
       <c r="W17">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\German_Aerospace_Center_DLR_C_Software_Developer_wmd_FSDM_and_HPC_Optimization.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\German_Aerospace_Center_DLR_C_Software_Developer_wmd_FSDM_and_HPC_Optimization.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X17">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\German_Aerospace_Center_DLR_C_Software_Developer_wmd_FSDM_and_HPC_Optimization.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\German_Aerospace_Center_DLR_C_Software_Developer_wmd_FSDM_and_HPC_Optimization.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y17">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\German_Aerospace_Center_DLR_C_Software_Developer_wmd_FSDM_and_HPC_Optimization_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\German_Aerospace_Center_DLR_C_Software_Developer_wmd_FSDM_and_HPC_Optimization_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:41.896498</t>
+          <t>2026-06-28T09:17:47.521824</t>
         </is>
       </c>
     </row>
@@ -2409,20 +2385,20 @@
         </is>
       </c>
       <c r="W18">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\ACONEXT_System_Engineer_Linux_HPC_mwd.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\ACONEXT_System_Engineer_Linux_HPC_mwd.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X18">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\ACONEXT_System_Engineer_Linux_HPC_mwd.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\ACONEXT_System_Engineer_Linux_HPC_mwd.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y18">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\ACONEXT_System_Engineer_Linux_HPC_mwd_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\ACONEXT_System_Engineer_Linux_HPC_mwd_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:41.976066</t>
+          <t>2026-06-28T09:17:47.564924</t>
         </is>
       </c>
     </row>
@@ -2478,11 +2454,7 @@
           <t>Quantum Computing, Physics, HPC, Python, Research, Optimization Methods</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>qiskit, cirq</t>
-        </is>
-      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>PhD Fellowship (Fall 2026)</t>
@@ -2504,11 +2476,11 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Overall match: 85%; Education: 70%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 40%; Strengths: Python programming, HPC background, Quantum computing knowledge, Optimization methods expertise; Missing: qiskit, cirq</t>
+          <t>Overall match: 88%; Education: 70%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 40%; Strengths: Python programming, HPC background, Quantum computing knowledge, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2522,20 +2494,20 @@
         </is>
       </c>
       <c r="W19">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Max_Planck_Institute_Munich_Quantum_Valley_IMPRS_Q_PhD_IMPRS_Doctoral_Fellowships_in_Quantum_Science_.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Max_Planck_Institute_Munich_Quantum_Valley_IMPRS_Q_PhD_IMPRS_Doctoral_Fellowships_in_Quantum_Science_.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X19">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Max_Planck_Institute_Munich_Quantum_Valley_IMPRS_Q_PhD_IMPRS_Doctoral_Fellowships_in_Quantum_Science_.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Max_Planck_Institute_Munich_Quantum_Valley_IMPRS_Q_PhD_IMPRS_Doctoral_Fellowships_in_Quantum_Science_.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y19">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Max_Planck_Institute_Munich_Quantum_Valley_IMPRS_Q_PhD_IMPRS_Doctoral_Fellowships_in_Quantum_Science__CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Max_Planck_Institute_Munich_Quantum_Valley_IMPRS_Q_PhD_IMPRS_Doctoral_Fellowships_in_Quantum_Science__CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:42.033673</t>
+          <t>2026-06-28T09:17:47.867502</t>
         </is>
       </c>
     </row>
@@ -2631,20 +2603,20 @@
         </is>
       </c>
       <c r="W20">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Forschungszentrum_Jülich_ICE_1_Master_Thesis_Hybrid_ML_LLM_based_Fault_Detection_.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Forschungszentrum_Jülich_ICE_1_Master_Thesis_Hybrid_ML_LLM_based_Fault_Detection_.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X20">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Forschungszentrum_Jülich_ICE_1_Master_Thesis_Hybrid_ML_LLM_based_Fault_Detection_.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Forschungszentrum_Jülich_ICE_1_Master_Thesis_Hybrid_ML_LLM_based_Fault_Detection_.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y20">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Forschungszentrum_Jülich_ICE_1_Master_Thesis_Hybrid_ML_LLM_based_Fault_Detection__CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Forschungszentrum_Jülich_ICE_1_Master_Thesis_Hybrid_ML_LLM_based_Fault_Detection__CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:42.156589</t>
+          <t>2026-06-28T09:17:47.902431</t>
         </is>
       </c>
     </row>
@@ -2884,11 +2856,7 @@
           <t>C++, HPC, GPU, Python, Scientific Software, Performance Optimization</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>cuda</t>
-        </is>
-      </c>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>Engineering</t>
@@ -2910,11 +2878,11 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Overall match: 79%; Education: 40%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: cuda</t>
+          <t>Overall match: 82%; Education: 40%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2928,20 +2896,20 @@
         </is>
       </c>
       <c r="W23">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\CERN_Software_Engineer_High_Performance_Computing_EP_SF.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\CERN_Software_Engineer_High_Performance_Computing_EP_SF.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X23">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\CERN_Software_Engineer_High_Performance_Computing_EP_SF.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\CERN_Software_Engineer_High_Performance_Computing_EP_SF.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y23">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\CERN_Software_Engineer_High_Performance_Computing_EP_SF_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\CERN_Software_Engineer_High_Performance_Computing_EP_SF_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:45.943867</t>
+          <t>2026-06-28T09:17:51.520419</t>
         </is>
       </c>
     </row>
@@ -3033,20 +3001,20 @@
         </is>
       </c>
       <c r="W24">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\CERN_Short_Term_Internship_2026_TechnicalComputing.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\CERN_Short_Term_Internship_2026_TechnicalComputing.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X24">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\CERN_Short_Term_Internship_2026_TechnicalComputing.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\CERN_Short_Term_Internship_2026_TechnicalComputing.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y24">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\CERN_Short_Term_Internship_2026_TechnicalComputing_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\CERN_Short_Term_Internship_2026_TechnicalComputing_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:46.047499</t>
+          <t>2026-06-28T09:17:51.751744</t>
         </is>
       </c>
     </row>
@@ -3142,20 +3110,20 @@
         </is>
       </c>
       <c r="W25">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\CERN_Openlab_CERN_Openlab_Summer_Student_Programme_2026.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\CERN_Openlab_CERN_Openlab_Summer_Student_Programme_2026.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X25">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\CERN_Openlab_CERN_Openlab_Summer_Student_Programme_2026.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\CERN_Openlab_CERN_Openlab_Summer_Student_Programme_2026.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y25">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\CERN_Openlab_CERN_Openlab_Summer_Student_Programme_2026_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\CERN_Openlab_CERN_Openlab_Summer_Student_Programme_2026_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:46.229113</t>
+          <t>2026-06-28T09:17:52.148363</t>
         </is>
       </c>
     </row>
@@ -3211,11 +3179,7 @@
           <t>Quantum Computing, Python, ML, Algorithms, Research</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>qiskit, cirq</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>Internship</t>
@@ -3237,11 +3201,11 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Overall match: 88%; Education: 70%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 70%; Strengths: Python programming, Quantum computing knowledge; Missing: qiskit, cirq</t>
+          <t>Overall match: 91%; Education: 70%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 70%; Strengths: Python programming, Quantum computing knowledge</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3255,20 +3219,20 @@
         </is>
       </c>
       <c r="W26">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Quantinuum_Internship_Opportunities_Quantum_Software_ML_Algor.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Quantinuum_Internship_Opportunities_Quantum_Software_ML_Algor.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X26">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Quantinuum_Internship_Opportunities_Quantum_Software_ML_Algor.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Quantinuum_Internship_Opportunities_Quantum_Software_ML_Algor.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y26">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Quantinuum_Internship_Opportunities_Quantum_Software_ML_Algor_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Quantinuum_Internship_Opportunities_Quantum_Software_ML_Algor_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:46.193313</t>
+          <t>2026-06-28T09:17:51.916490</t>
         </is>
       </c>
     </row>
@@ -3364,20 +3328,20 @@
         </is>
       </c>
       <c r="W27">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\EUMaster4HPC_Consortium_Masters_Thesis_Internship_Multiple_EU_Locations.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\EUMaster4HPC_Consortium_Masters_Thesis_Internship_Multiple_EU_Locations.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X27">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\EUMaster4HPC_Consortium_Masters_Thesis_Internship_Multiple_EU_Locations.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\EUMaster4HPC_Consortium_Masters_Thesis_Internship_Multiple_EU_Locations.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y27">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\EUMaster4HPC_Consortium_Masters_Thesis_Internship_Multiple_EU_Locations_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\EUMaster4HPC_Consortium_Masters_Thesis_Internship_Multiple_EU_Locations_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:49.971195</t>
+          <t>2026-06-28T09:17:55.530059</t>
         </is>
       </c>
     </row>
@@ -3455,11 +3419,11 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Overall match: 90%; Education: 80%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background</t>
+          <t>Overall match: 93%; Education: 80%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3473,20 +3437,20 @@
         </is>
       </c>
       <c r="W28">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\EUMaster4HPC_EuroHPC_JU_Partners_Research_Internship_Master_Thesis_at_EuroHPC_JU_Pa.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\EUMaster4HPC_EuroHPC_JU_Partners_Research_Internship_Master_Thesis_at_EuroHPC_JU_Pa.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X28">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\EUMaster4HPC_EuroHPC_JU_Partners_Research_Internship_Master_Thesis_at_EuroHPC_JU_Pa.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\EUMaster4HPC_EuroHPC_JU_Partners_Research_Internship_Master_Thesis_at_EuroHPC_JU_Pa.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y28">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\EUMaster4HPC_EuroHPC_JU_Partners_Research_Internship_Master_Thesis_at_EuroHPC_JU_Pa_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\EUMaster4HPC_EuroHPC_JU_Partners_Research_Internship_Master_Thesis_at_EuroHPC_JU_Pa_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:50.062398</t>
+          <t>2026-06-28T09:17:55.704053</t>
         </is>
       </c>
     </row>
@@ -3542,11 +3506,7 @@
           <t>HPC, GPU, PhD, Research, Python, C</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>mpi, cuda</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>PhD</t>
@@ -3568,11 +3528,11 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Overall match: 88%; Education: 70%, Skills: 100%, Programming: 100%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, cuda</t>
+          <t>Overall match: 91%; Education: 70%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background, Optimization methods expertise</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3586,20 +3546,20 @@
         </is>
       </c>
       <c r="W29">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\HiPEAC_Network_Various_Partners_PhD_Student_HPC_GPU_Computing.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\HiPEAC_Network_Various_Partners_PhD_Student_HPC_GPU_Computing.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X29">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\HiPEAC_Network_Various_Partners_PhD_Student_HPC_GPU_Computing.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\HiPEAC_Network_Various_Partners_PhD_Student_HPC_GPU_Computing.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y29">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\HiPEAC_Network_Various_Partners_PhD_Student_HPC_GPU_Computing_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\HiPEAC_Network_Various_Partners_PhD_Student_HPC_GPU_Computing_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:50.674660</t>
+          <t>2026-06-28T09:17:55.934340</t>
         </is>
       </c>
     </row>
@@ -3769,11 +3729,11 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Overall match: 69%; Education: 70%, Skills: 60%, Programming: 100%; Research: 80%, Experience: 40%; Strengths: Python programming</t>
+          <t>Overall match: 88%; Education: 70%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 40%; Strengths: Python programming</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3787,20 +3747,20 @@
         </is>
       </c>
       <c r="W31">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\University_of_Innsbruck_UIBK_PhD_Positions_in_AI_Driven_Edge_Cloud_Computing.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\University_of_Innsbruck_UIBK_PhD_Positions_in_AI_Driven_Edge_Cloud_Computing.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X31">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\University_of_Innsbruck_UIBK_PhD_Positions_in_AI_Driven_Edge_Cloud_Computing.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\University_of_Innsbruck_UIBK_PhD_Positions_in_AI_Driven_Edge_Cloud_Computing.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y31">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\University_of_Innsbruck_UIBK_PhD_Positions_in_AI_Driven_Edge_Cloud_Computing_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\University_of_Innsbruck_UIBK_PhD_Positions_in_AI_Driven_Edge_Cloud_Computing_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:50.515002</t>
+          <t>2026-06-28T09:17:56.039009</t>
         </is>
       </c>
     </row>
@@ -3878,11 +3838,11 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Overall match: 74%; Education: 40%, Skills: 80%, Programming: 100%; Research: 80%, Experience: 70%; Strengths: Python programming, HPC background</t>
+          <t>Overall match: 85%; Education: 40%, Skills: 100%, Programming: 100%; Research: 100%, Experience: 70%; Strengths: Python programming, HPC background</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3896,20 +3856,20 @@
         </is>
       </c>
       <c r="W32">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\University_of_Torino_ICSC_Italian_National_Center__Postdoc_in_Parallel_and_Distributed_Computing_Clou.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\University_of_Torino_ICSC_Italian_National_Center__Postdoc_in_Parallel_and_Distributed_Computing_Clou.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X32">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\University_of_Torino_ICSC_Italian_National_Center__Postdoc_in_Parallel_and_Distributed_Computing_Clou.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\University_of_Torino_ICSC_Italian_National_Center__Postdoc_in_Parallel_and_Distributed_Computing_Clou.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y32">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\University_of_Torino_ICSC_Italian_National_Center__Postdoc_in_Parallel_and_Distributed_Computing_Clou_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\University_of_Torino_ICSC_Italian_National_Center__Postdoc_in_Parallel_and_Distributed_Computing_Clou_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:54.141854</t>
+          <t>2026-06-28T09:17:59.671210</t>
         </is>
       </c>
     </row>
@@ -3987,11 +3947,11 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="n">
-        <v>72.2</v>
+        <v>75.2</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Overall match: 72%; Education: 40%, Skills: 100%, Programming: 55%; Research: 80%, Experience: 40%; Strengths: Python programming, Quantum computing knowledge</t>
+          <t>Overall match: 75%; Education: 40%, Skills: 100%, Programming: 55%; Research: 100%, Experience: 40%; Strengths: Python programming, Quantum computing knowledge</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4005,20 +3965,20 @@
         </is>
       </c>
       <c r="W33">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\University_of_Applied_Sciences_and_Arts_of_Western_Postdoctoral_Researcher_in_Applied_Research_in_Pos.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\University_of_Applied_Sciences_and_Arts_of_Western_Postdoctoral_Researcher_in_Applied_Research_in_Pos.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X33">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\University_of_Applied_Sciences_and_Arts_of_Western_Postdoctoral_Researcher_in_Applied_Research_in_Pos.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\University_of_Applied_Sciences_and_Arts_of_Western_Postdoctoral_Researcher_in_Applied_Research_in_Pos.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y33">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\University_of_Applied_Sciences_and_Arts_of_Western_Postdoctoral_Researcher_in_Applied_Research_in_Pos_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\University_of_Applied_Sciences_and_Arts_of_Western_Postdoctoral_Researcher_in_Applied_Research_in_Pos_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:54.355101</t>
+          <t>2026-06-28T09:17:59.793678</t>
         </is>
       </c>
     </row>
@@ -4444,7 +4404,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>mpi, aws, azure</t>
+          <t>aws, azure</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4468,11 +4428,11 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
-        <v>78.5</v>
+        <v>82.5</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Overall match: 78%; Education: 50%, Skills: 90%, Programming: 100%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: mpi, aws, azure</t>
+          <t>Overall match: 82%; Education: 50%, Skills: 100%, Programming: 100%; Research: 90%, Experience: 40%; Strengths: Python programming, HPC background, Optimization methods expertise; Missing: aws, azure</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4486,20 +4446,20 @@
         </is>
       </c>
       <c r="W38">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\HMx_Labs_HPC_Software_Engineer.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\HMx_Labs_HPC_Software_Engineer.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X38">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\HMx_Labs_HPC_Software_Engineer.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\HMx_Labs_HPC_Software_Engineer.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y38">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\HMx_Labs_HPC_Software_Engineer_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\HMx_Labs_HPC_Software_Engineer_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:54.425388</t>
+          <t>2026-06-28T09:18:00.056987</t>
         </is>
       </c>
     </row>
@@ -4925,7 +4885,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>cuda, kubernetes</t>
+          <t>kubernetes</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4949,11 +4909,11 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="n">
-        <v>71.5</v>
+        <v>79.5</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>Overall match: 72%; Education: 50%, Skills: 80%, Programming: 100%; Research: 70%, Experience: 40%; Strengths: Python programming, HPC background; Missing: cuda, kubernetes</t>
+          <t>Overall match: 80%; Education: 50%, Skills: 100%, Programming: 100%; Research: 70%, Experience: 40%; Strengths: Python programming, HPC background; Missing: kubernetes</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -4967,20 +4927,20 @@
         </is>
       </c>
       <c r="W43">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\tex\Alpha_Compute_Corp_Lead_GPU_Infrastructure_Engineer_HPC_Fleet.tex","Open Resume Tex")</f>
+        <f>HYPERLINK("generated\CV\tex\Alpha_Compute_Corp_Lead_GPU_Infrastructure_Engineer_HPC_Fleet.tex","Open Resume Tex")</f>
         <v/>
       </c>
       <c r="X43">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CV\pdf\Alpha_Compute_Corp_Lead_GPU_Infrastructure_Engineer_HPC_Fleet.pdf","Open Resume Pdf")</f>
+        <f>HYPERLINK("generated\CV\pdf\Alpha_Compute_Corp_Lead_GPU_Infrastructure_Engineer_HPC_Fleet.pdf","Open Resume Pdf")</f>
         <v/>
       </c>
       <c r="Y43">
-        <f>HYPERLINK("C:\Users\ASWA\Music\Playlists\project Job\generated\CoverLetters\docx\Alpha_Compute_Corp_Lead_GPU_Infrastructure_Engineer_HPC_Fleet_CoverLetter.docx","Open Cover Letter")</f>
+        <f>HYPERLINK("generated\CoverLetters\docx\Alpha_Compute_Corp_Lead_GPU_Infrastructure_Engineer_HPC_Fleet_CoverLetter.docx","Open Cover Letter")</f>
         <v/>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>2026-06-27T20:41:54.539466</t>
+          <t>2026-06-28T09:18:00.082178</t>
         </is>
       </c>
     </row>

</xml_diff>